<commit_message>
Hogar de Refugio: equipamiento y mobiliario listo para imprimir
Índice lleno en los Word (indice_word.py), edificaciones E-06 a E-08 como Habitaciones y cotejo de
cantidades entre metrado, especificaciones y memoria.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_EQUIPAMIENTO_Y_MOBILIARIO_HOGAR_REFUGIO.xlsx
+++ b/entregables/METRADO_EQUIPAMIENTO_Y_MOBILIARIO_HOGAR_REFUGIO.xlsx
@@ -11059,7 +11059,7 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>E-06  Dormitorios (1) - HABITACIONES ESPECIAL, DOBLES Y SIMPLES</t>
+          <t>E-06  Habitaciones (1) - HABITACIONES ESPECIAL, DOBLES Y SIMPLES</t>
         </is>
       </c>
       <c r="B198" s="4" t="n"/>
@@ -11312,7 +11312,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>E-06  Dormitorios (1) - SS.HH. DE LAS HABITACIONES</t>
+          <t>E-06  Habitaciones (1) - SS.HH. DE LAS HABITACIONES</t>
         </is>
       </c>
       <c r="B205" s="4" t="n"/>
@@ -11445,7 +11445,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>E-07  Dormitorios (2) - HABITACIONES ESPECIAL, DOBLES Y SIMPLES</t>
+          <t>E-07  Habitaciones (2) - HABITACIONES ESPECIAL, DOBLES Y SIMPLES</t>
         </is>
       </c>
       <c r="B209" s="4" t="n"/>
@@ -11738,7 +11738,7 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>E-07  Dormitorios (2) - SS.HH. DE LAS HABITACIONES</t>
+          <t>E-07  Habitaciones (2) - SS.HH. DE LAS HABITACIONES</t>
         </is>
       </c>
       <c r="B217" s="4" t="n"/>
@@ -11871,7 +11871,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>E-08  Dormitorios (3) - HABITACIONES ESPECIAL, DOBLES Y SIMPLES</t>
+          <t>E-08  Habitaciones (3) - HABITACIONES ESPECIAL, DOBLES Y SIMPLES</t>
         </is>
       </c>
       <c r="B221" s="4" t="n"/>
@@ -12124,7 +12124,7 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>E-08  Dormitorios (3) - SS.HH. DE LAS HABITACIONES</t>
+          <t>E-08  Habitaciones (3) - SS.HH. DE LAS HABITACIONES</t>
         </is>
       </c>
       <c r="B228" s="4" t="n"/>

</xml_diff>